<commit_message>
edited code so SR_Data_editsv2 spreadsheet now used
</commit_message>
<xml_diff>
--- a/survey_wqdata/SR_Data_editsv2.xlsx
+++ b/survey_wqdata/SR_Data_editsv2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atweg\Documents\Mike\Nokuse\charli_2025-11-03_email_surveydata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atweg\Documents\Mike\Nokuse\R_sevensrun\nokuse_seven_runs_survey\survey_wqdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD76E60C-E348-48B9-878A-63334F585356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADFAE02-DFDF-4877-923B-AC1E4FCADF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
   </bookViews>
@@ -238,6 +238,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -282,12 +285,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -625,1907 +633,1913 @@
   <dimension ref="A1:AD21"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="10.28515625" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="11.140625" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" customWidth="1"/>
-    <col min="16" max="16" width="12.28515625" customWidth="1"/>
-    <col min="17" max="18" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="8.76171875" style="5"/>
+    <col min="3" max="3" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.80859375" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" style="9" customWidth="1"/>
+    <col min="6" max="8" width="11.85546875" style="9" customWidth="1"/>
+    <col min="10" max="10" width="8.76171875" style="9"/>
+    <col min="11" max="11" width="10.28515625" style="9" customWidth="1"/>
+    <col min="12" max="12" width="8.76171875" style="9"/>
+    <col min="13" max="13" width="14" style="9" customWidth="1"/>
+    <col min="14" max="14" width="11.140625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="9" customWidth="1"/>
+    <col min="16" max="16" width="12.28515625" style="9" customWidth="1"/>
+    <col min="17" max="17" width="10.7109375" style="9" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" style="5" customWidth="1"/>
+    <col min="19" max="22" width="8.76171875" style="9"/>
+    <col min="23" max="30" width="8.76171875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>55</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="T1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="V1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:30">
-      <c r="A2" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C2" s="2">
         <v>45909</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="8">
         <v>0.5</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="9">
         <v>30.576194999999998</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="9">
         <v>-86.038640000000001</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="9">
         <v>30.576194999999998</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="9">
         <v>-86.038640000000001</v>
       </c>
       <c r="I2" t="s">
         <v>39</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="9">
         <v>0.25</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="9">
         <v>22.7</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="9">
         <v>5.08</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="9">
         <v>7.71</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="9">
         <v>89.5</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="9">
         <v>17.600000000000001</v>
       </c>
-      <c r="P2">
+      <c r="P2" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q2">
+      <c r="Q2" s="9">
         <v>1.63</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S2">
+      <c r="S2" s="9">
         <v>1.37</v>
       </c>
-      <c r="T2">
+      <c r="T2" s="9">
         <v>1.63</v>
       </c>
-      <c r="U2">
+      <c r="U2" s="9">
         <v>0.34</v>
       </c>
-      <c r="V2">
+      <c r="V2" s="9">
         <v>99.48</v>
       </c>
-      <c r="W2" t="s">
-        <v>35</v>
-      </c>
-      <c r="X2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y2" t="s">
+      <c r="W2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="Z2" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD2" t="s">
+      <c r="AA2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD2" s="5" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" t="s">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C3" s="2">
         <v>45909</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="9">
         <v>30.574836999999999</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="9">
         <v>-86.028282000000004</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="9">
         <v>30.574836999999999</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="9">
         <v>-86.028282000000004</v>
       </c>
       <c r="I3" t="s">
         <v>39</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="9">
         <v>0.38</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="9">
         <v>25.6</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="9">
         <v>5.39</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="9">
         <v>7.93</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="9">
         <v>97.1</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="9">
         <v>18.100000000000001</v>
       </c>
-      <c r="P3">
+      <c r="P3" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="9">
         <v>2.56</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S3">
+      <c r="S3" s="9">
         <v>2.69</v>
       </c>
-      <c r="T3">
+      <c r="T3" s="9">
         <v>2.9</v>
       </c>
-      <c r="U3">
+      <c r="U3" s="9">
         <v>0.13</v>
       </c>
-      <c r="V3">
+      <c r="V3" s="9">
         <v>95.84</v>
       </c>
-      <c r="W3" t="s">
-        <v>35</v>
-      </c>
-      <c r="X3" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y3" t="s">
+      <c r="W3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="Z3" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA3" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC3" t="s">
+      <c r="AA3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC3" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:30">
-      <c r="A4" t="s">
+      <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="2">
         <v>45909</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="8">
         <v>0.44930555555555557</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="9">
         <v>30.568359999999998</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="9">
         <v>-86.016197000000005</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="9">
         <v>30.568359999999998</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="9">
         <v>-86.016197000000005</v>
       </c>
       <c r="I4" t="s">
         <v>39</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="9">
         <v>0.4</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="9">
         <v>22.5</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="9">
         <v>5.01</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="9">
         <v>8.0299999999999994</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="9">
         <v>92.7</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="9">
         <v>19.100000000000001</v>
       </c>
-      <c r="P4">
+      <c r="P4" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="9">
         <v>2.14</v>
       </c>
-      <c r="R4" t="s">
+      <c r="R4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S4">
+      <c r="S4" s="9">
         <v>4.83</v>
       </c>
-      <c r="T4">
+      <c r="T4" s="9">
         <v>6.04</v>
       </c>
-      <c r="U4">
+      <c r="U4" s="9">
         <v>0.27</v>
       </c>
-      <c r="V4">
+      <c r="V4" s="9">
         <v>99.48</v>
       </c>
-      <c r="W4" t="s">
-        <v>35</v>
-      </c>
-      <c r="X4" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y4" t="s">
+      <c r="W4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="Z4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA4" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD4" t="s">
+      <c r="AA4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD4" s="5" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:30">
-      <c r="A5" t="s">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C5" s="2">
         <v>45912</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="8">
         <v>0.3840277777777778</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="9">
         <v>30.558720000000001</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="9">
         <v>-85.978043</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="9">
         <v>30.558720000000001</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="9">
         <v>-85.978043</v>
       </c>
       <c r="I5" t="s">
         <v>39</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="9">
         <v>0.32</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="9">
         <v>20.6</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="9">
         <v>5.64</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="9">
         <v>8.4700000000000006</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="9">
         <v>94.4</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="9">
         <v>19.100000000000001</v>
       </c>
-      <c r="P5">
+      <c r="P5" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="9">
         <v>2.5099999999999998</v>
       </c>
-      <c r="R5" t="s">
+      <c r="R5" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S5">
+      <c r="S5" s="9">
         <v>6.45</v>
       </c>
-      <c r="T5">
+      <c r="T5" s="9">
         <v>7.06</v>
       </c>
-      <c r="U5">
+      <c r="U5" s="9">
         <v>0.37</v>
       </c>
-      <c r="V5">
+      <c r="V5" s="9">
         <v>84.92</v>
       </c>
-      <c r="W5" t="s">
-        <v>35</v>
-      </c>
-      <c r="X5" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y5" t="s">
+      <c r="W5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="Z5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA5" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC5" t="s">
+      <c r="AA5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC5" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:30">
-      <c r="A6" t="s">
+      <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="2">
         <v>45911</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="9">
         <v>30.556989999999999</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="9">
         <v>-85.963539999999995</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="9">
         <v>30.556778000000001</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="9">
         <v>-85.963860999999994</v>
       </c>
       <c r="I6" t="s">
         <v>39</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="9">
         <v>0.32</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="9">
         <v>21.8</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="9">
         <v>5.55</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="9">
         <v>8.33</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="9">
         <v>94.9</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="9">
         <v>19.100000000000001</v>
       </c>
-      <c r="P6">
+      <c r="P6" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q6">
+      <c r="Q6" s="9">
         <v>3.71</v>
       </c>
-      <c r="R6" t="s">
+      <c r="R6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S6">
+      <c r="S6" s="9">
         <v>5.13</v>
       </c>
-      <c r="T6">
+      <c r="T6" s="9">
         <v>6.37</v>
       </c>
-      <c r="U6">
+      <c r="U6" s="9">
         <v>0.41</v>
       </c>
-      <c r="V6">
+      <c r="V6" s="9">
         <v>96.1</v>
       </c>
-      <c r="W6" t="s">
-        <v>35</v>
-      </c>
-      <c r="X6" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y6" t="s">
+      <c r="W6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="Z6" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA6" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC6" t="s">
+      <c r="AA6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC6" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:30">
-      <c r="A7" t="s">
+      <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="2">
         <v>45911</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="8">
         <v>0.53541666666666665</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="9">
         <v>30.557153</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="9">
         <v>-85.962569000000002</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="9">
         <v>30.557153</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="9">
         <v>-85.962569000000002</v>
       </c>
       <c r="I7" t="s">
         <v>39</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="9">
         <v>0.43</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="9">
         <v>21.6</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="9">
         <v>5.6</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="9">
         <v>8.3000000000000007</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="9">
         <v>94.2</v>
       </c>
-      <c r="O7">
+      <c r="O7" s="9">
         <v>19.100000000000001</v>
       </c>
-      <c r="P7">
+      <c r="P7" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="9">
         <v>2.33</v>
       </c>
-      <c r="R7" t="s">
+      <c r="R7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S7">
+      <c r="S7" s="9">
         <v>4.83</v>
       </c>
-      <c r="T7">
+      <c r="T7" s="9">
         <v>6.81</v>
       </c>
-      <c r="U7">
+      <c r="U7" s="9">
         <v>0.71</v>
       </c>
-      <c r="V7">
+      <c r="V7" s="9">
         <v>92.72</v>
       </c>
-      <c r="W7" t="s">
-        <v>35</v>
-      </c>
-      <c r="X7" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y7" t="s">
+      <c r="W7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y7" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="Z7" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA7" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC7" t="s">
+      <c r="AA7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC7" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:30">
-      <c r="A8" t="s">
+      <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C8" s="2">
         <v>45910</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="8">
         <v>0.37986111111111109</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="9">
         <v>30.581834000000001</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="9">
         <v>-85.979294999999993</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="9">
         <v>30.581028</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="9">
         <v>-85.979388999999998</v>
       </c>
       <c r="I8" t="s">
         <v>39</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="9">
         <v>0.32</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="9">
         <v>21.9</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="9">
         <v>6.32</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="9">
         <v>7.68</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="9">
         <v>87.7</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="9">
         <v>39.200000000000003</v>
       </c>
-      <c r="P8">
+      <c r="P8" s="9">
         <v>0.02</v>
       </c>
-      <c r="Q8">
+      <c r="Q8" s="9">
         <v>1.44</v>
       </c>
-      <c r="R8" t="s">
+      <c r="R8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S8">
+      <c r="S8" s="9">
         <v>1.65</v>
       </c>
-      <c r="T8">
+      <c r="T8" s="9">
         <v>2.36</v>
       </c>
-      <c r="U8">
+      <c r="U8" s="9">
         <v>0.06</v>
       </c>
-      <c r="V8">
+      <c r="V8" s="9">
         <v>97.92</v>
       </c>
-      <c r="W8" t="s">
-        <v>35</v>
-      </c>
-      <c r="X8" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y8" t="s">
+      <c r="W8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y8" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="Z8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC8" t="s">
+      <c r="AA8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC8" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:30">
-      <c r="A9" t="s">
+      <c r="A9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C9" s="2">
         <v>45910</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="8">
         <v>0.39791666666666664</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="9">
         <v>30.579967</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="9">
         <v>-85.980097000000001</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="9">
         <v>30.579861000000001</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="9">
         <v>-85.979889</v>
       </c>
       <c r="I9" t="s">
         <v>39</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="9">
         <v>0.25</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="9">
         <v>21.9</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="9">
         <v>6.39</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="9">
         <v>7.94</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="9">
         <v>90.7</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="9">
         <v>38.4</v>
       </c>
-      <c r="P9">
+      <c r="P9" s="9">
         <v>0.02</v>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="9">
         <v>1.74</v>
       </c>
-      <c r="R9" t="s">
+      <c r="R9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S9">
+      <c r="S9" s="9">
         <v>1.0900000000000001</v>
       </c>
-      <c r="T9">
+      <c r="T9" s="9">
         <v>1.83</v>
       </c>
-      <c r="U9">
+      <c r="U9" s="9">
         <v>0.08</v>
       </c>
-      <c r="V9">
+      <c r="V9" s="9">
         <v>100</v>
       </c>
-      <c r="W9" t="s">
-        <v>35</v>
-      </c>
-      <c r="X9" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y9" t="s">
+      <c r="W9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="Z9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA9" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC9" t="s">
+      <c r="AA9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC9" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:30">
-      <c r="A10" t="s">
+      <c r="A10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C10" s="2">
         <v>45910</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="8">
         <v>0.52152777777777781</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="9">
         <v>30.569496000000001</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="9">
         <v>-85.979523</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="9">
         <v>30.569500000000001</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="9">
         <v>-85.979528000000002</v>
       </c>
       <c r="I10" t="s">
         <v>39</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="9">
         <v>0.25</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="9">
         <v>22.6</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="9">
         <v>6.37</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="9">
         <v>7.69</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="9">
         <v>89.1</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="9">
         <v>22.2</v>
       </c>
-      <c r="P10">
+      <c r="P10" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="9">
         <v>2.2999999999999998</v>
       </c>
-      <c r="R10" t="s">
+      <c r="R10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S10">
+      <c r="S10" s="9">
         <v>2.82</v>
       </c>
-      <c r="T10">
+      <c r="T10" s="9">
         <v>3.56</v>
       </c>
-      <c r="U10">
+      <c r="U10" s="9">
         <v>0.22</v>
       </c>
-      <c r="V10">
+      <c r="V10" s="9">
         <v>98.18</v>
       </c>
-      <c r="W10" t="s">
-        <v>35</v>
-      </c>
-      <c r="X10" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y10" t="s">
+      <c r="W10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y10" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="Z10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA10" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB10" t="s">
+      <c r="AA10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB10" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="AC10" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD10" t="s">
+      <c r="AC10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD10" s="5" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:30">
-      <c r="A11" t="s">
+      <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C11" s="2">
         <v>45910</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="9">
         <v>30.567005999999999</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="9">
         <f>F29-85.979297</f>
         <v>-85.979297000000003</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="9">
         <v>30.566330000000001</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="9">
         <v>-85.97851</v>
       </c>
       <c r="I11" t="s">
         <v>39</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="9">
         <v>0.34</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="9">
         <v>23</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="9">
         <v>5.86</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="9">
         <v>7.65</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="9">
         <v>89.1</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="9">
         <v>22.1</v>
       </c>
-      <c r="P11">
+      <c r="P11" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="9">
         <v>3.08</v>
       </c>
-      <c r="R11" t="s">
+      <c r="R11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S11">
+      <c r="S11" s="9">
         <v>2.11</v>
       </c>
-      <c r="T11">
+      <c r="T11" s="9">
         <v>3.25</v>
       </c>
-      <c r="U11">
+      <c r="U11" s="9">
         <v>0.13</v>
       </c>
-      <c r="V11">
+      <c r="V11" s="9">
         <v>98.44</v>
       </c>
-      <c r="W11" t="s">
-        <v>35</v>
-      </c>
-      <c r="X11" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y11" t="s">
+      <c r="W11" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X11" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y11" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z11" t="s">
+      <c r="Z11" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA11" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB11" t="s">
+      <c r="AA11" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB11" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="AC11" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD11" t="s">
+      <c r="AC11" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD11" s="5" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:30">
-      <c r="A12" t="s">
+      <c r="A12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C12" s="2">
         <v>45910</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="8">
         <v>0.43472222222222223</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="9">
         <v>30.580921</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="9">
         <v>-85.964935999999994</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="9">
         <v>30.580943999999999</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="9">
         <v>-85.965056000000004</v>
       </c>
       <c r="I12" t="s">
         <v>39</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="9">
         <v>0.23</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="9">
         <v>22</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="9">
         <v>4.82</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="9">
         <v>7.02</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="9">
         <v>80.400000000000006</v>
       </c>
-      <c r="O12">
+      <c r="O12" s="9">
         <v>22.6</v>
       </c>
-      <c r="P12">
+      <c r="P12" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="9">
         <v>2</v>
       </c>
-      <c r="R12" t="s">
+      <c r="R12" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S12">
+      <c r="S12" s="9">
         <v>1.4</v>
       </c>
-      <c r="T12">
+      <c r="T12" s="9">
         <v>2</v>
       </c>
-      <c r="U12">
+      <c r="U12" s="9">
         <v>0.13</v>
       </c>
-      <c r="V12">
+      <c r="V12" s="9">
         <v>99.22</v>
       </c>
-      <c r="W12" t="s">
-        <v>35</v>
-      </c>
-      <c r="X12" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y12" t="s">
+      <c r="W12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z12" t="s">
+      <c r="Z12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA12" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB12" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC12" t="s">
+      <c r="AA12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC12" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:30">
-      <c r="A13" t="s">
+      <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="2">
         <v>45910</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="8">
         <v>0.4777777777777778</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="9">
         <v>30.570474999999998</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="9">
         <v>-85.966836999999998</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="9">
         <v>30.570471999999999</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="9">
         <v>-85.966333000000006</v>
       </c>
       <c r="I13" t="s">
         <v>39</v>
       </c>
-      <c r="J13">
+      <c r="J13" s="9">
         <v>0.31</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="9">
         <v>22.6</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="9">
         <v>5.0199999999999996</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="9">
         <v>7.17</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="9">
         <v>83</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="9">
         <v>20.2</v>
       </c>
-      <c r="P13">
+      <c r="P13" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q13">
+      <c r="Q13" s="9">
         <v>2.48</v>
       </c>
-      <c r="R13" t="s">
+      <c r="R13" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S13">
+      <c r="S13" s="9">
         <v>2.74</v>
       </c>
-      <c r="T13">
+      <c r="T13" s="9">
         <v>2.85</v>
       </c>
-      <c r="U13">
+      <c r="U13" s="9">
         <v>0.2</v>
       </c>
-      <c r="V13">
+      <c r="V13" s="9">
         <v>99.48</v>
       </c>
-      <c r="W13" t="s">
-        <v>35</v>
-      </c>
-      <c r="X13" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y13" t="s">
+      <c r="W13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z13" t="s">
+      <c r="Z13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA13" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB13" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC13" t="s">
+      <c r="AA13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC13" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:30">
-      <c r="A14" t="s">
+      <c r="A14" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="2">
         <v>45911</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="8">
         <v>0.38055555555555554</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="9">
         <v>30.563506</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="9">
         <v>-85.966802999999999</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="9">
         <v>30.56325</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="9">
         <v>-85.966443999999996</v>
       </c>
       <c r="I14" t="s">
         <v>39</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="9">
         <v>0.3</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="9">
         <v>20.8</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="9">
         <v>5.0999999999999996</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="9">
         <v>7.78</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="9">
         <v>87.1</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="9">
         <v>19.899999999999999</v>
       </c>
-      <c r="P14">
+      <c r="P14" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q14">
+      <c r="Q14" s="9">
         <v>1.85</v>
       </c>
-      <c r="R14" t="s">
+      <c r="R14" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S14">
+      <c r="S14" s="9">
         <v>2.62</v>
       </c>
-      <c r="T14">
+      <c r="T14" s="9">
         <v>3</v>
       </c>
-      <c r="U14">
+      <c r="U14" s="9">
         <v>0.38</v>
       </c>
-      <c r="V14">
+      <c r="V14" s="9">
         <v>97.66</v>
       </c>
-      <c r="W14" t="s">
-        <v>35</v>
-      </c>
-      <c r="X14" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y14" t="s">
+      <c r="W14" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X14" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z14" t="s">
+      <c r="Z14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA14" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB14" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC14" t="s">
+      <c r="AA14" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB14" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC14" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:30">
-      <c r="A15" t="s">
+      <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="2">
         <v>45912</v>
       </c>
-      <c r="D15" s="3"/>
-      <c r="E15">
+      <c r="E15" s="9">
         <v>30.548777000000001</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="9">
         <v>-85.984607999999994</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="9">
         <v>30.548777000000001</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="9">
         <v>-85.984607999999994</v>
       </c>
       <c r="I15" t="s">
         <v>39</v>
       </c>
-      <c r="J15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K15" t="s">
-        <v>42</v>
-      </c>
-      <c r="L15" t="s">
-        <v>42</v>
-      </c>
-      <c r="M15" t="s">
-        <v>42</v>
-      </c>
-      <c r="N15" t="s">
-        <v>42</v>
-      </c>
-      <c r="O15" t="s">
-        <v>42</v>
-      </c>
-      <c r="P15" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>42</v>
-      </c>
-      <c r="R15" t="s">
-        <v>42</v>
-      </c>
-      <c r="S15" t="s">
-        <v>42</v>
-      </c>
-      <c r="T15" t="s">
-        <v>42</v>
-      </c>
-      <c r="U15" t="s">
-        <v>42</v>
-      </c>
-      <c r="V15" t="s">
-        <v>42</v>
-      </c>
-      <c r="W15" t="s">
-        <v>42</v>
-      </c>
-      <c r="X15" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y15" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z15" t="s">
-        <v>42</v>
-      </c>
-      <c r="AA15" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB15" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC15" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD15" t="s">
+      <c r="J15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="M15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="N15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="O15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="R15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="S15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="T15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="U15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="V15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="W15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD15" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:30">
-      <c r="A16" t="s">
+      <c r="A16" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C16" s="2">
         <v>45912</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="8">
         <v>0.3659722222222222</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="9">
         <v>30.557362000000001</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="9">
         <v>-85.981594000000001</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="9">
         <v>30.557362000000001</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="9">
         <v>-85.981594000000001</v>
       </c>
       <c r="I16" t="s">
         <v>39</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="9">
         <v>0.22</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="9">
         <v>20.7</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="9">
         <v>5.94</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="9">
         <v>8.58</v>
       </c>
-      <c r="N16">
+      <c r="N16" s="9">
         <v>95.6</v>
       </c>
-      <c r="O16">
+      <c r="O16" s="9">
         <v>21.9</v>
       </c>
-      <c r="P16">
+      <c r="P16" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q16">
+      <c r="Q16" s="9">
         <v>3.51</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R16" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S16">
+      <c r="S16" s="9">
         <v>2.72</v>
       </c>
-      <c r="T16">
+      <c r="T16" s="9">
         <v>2.97</v>
       </c>
-      <c r="U16">
+      <c r="U16" s="9">
         <v>0.41</v>
       </c>
-      <c r="V16">
+      <c r="V16" s="9">
         <v>98.18</v>
       </c>
-      <c r="W16" t="s">
-        <v>35</v>
-      </c>
-      <c r="X16" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y16" t="s">
+      <c r="W16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y16" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z16" t="s">
+      <c r="Z16" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA16" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB16" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC16" t="s">
+      <c r="AA16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB16" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC16" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:30">
-      <c r="A17" t="s">
+      <c r="A17" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C17" s="2">
         <v>45911</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="8">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="9">
         <v>30.549496000000001</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="9">
         <v>-85.919370000000001</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="9">
         <v>30.549496000000001</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="9">
         <v>-85.919370000000001</v>
       </c>
       <c r="I17" t="s">
         <v>39</v>
       </c>
-      <c r="J17" t="s">
-        <v>42</v>
-      </c>
-      <c r="K17" t="s">
-        <v>42</v>
-      </c>
-      <c r="L17" t="s">
-        <v>42</v>
-      </c>
-      <c r="M17" t="s">
-        <v>42</v>
-      </c>
-      <c r="N17" t="s">
-        <v>42</v>
-      </c>
-      <c r="O17" t="s">
-        <v>42</v>
-      </c>
-      <c r="P17" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>42</v>
-      </c>
-      <c r="R17" t="s">
-        <v>42</v>
-      </c>
-      <c r="S17" t="s">
-        <v>42</v>
-      </c>
-      <c r="T17" t="s">
-        <v>42</v>
-      </c>
-      <c r="U17" t="s">
-        <v>42</v>
-      </c>
-      <c r="V17" t="s">
-        <v>42</v>
-      </c>
-      <c r="W17" t="s">
-        <v>42</v>
-      </c>
-      <c r="X17" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y17" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z17" t="s">
-        <v>42</v>
-      </c>
-      <c r="AA17" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB17" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC17" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD17" t="s">
+      <c r="J17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="M17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="N17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="O17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="S17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="T17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="U17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="V17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="W17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD17" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:30">
-      <c r="A18" t="s">
+      <c r="A18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C18" s="2">
         <v>45909</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="8">
         <v>0.38333333333333336</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="9">
         <v>30.578201</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="9">
         <v>-85.999088</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="9">
         <v>30.578201</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="9">
         <v>-85.999088</v>
       </c>
       <c r="I18" t="s">
         <v>39</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="9">
         <v>0.36</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="9">
         <v>22.3</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="9">
         <v>4.8600000000000003</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="9">
         <v>7.63</v>
       </c>
-      <c r="N18">
+      <c r="N18" s="9">
         <v>88</v>
       </c>
-      <c r="O18">
+      <c r="O18" s="9">
         <v>21.6</v>
       </c>
-      <c r="P18">
+      <c r="P18" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q18">
+      <c r="Q18" s="9">
         <v>2.82</v>
       </c>
-      <c r="R18" t="s">
+      <c r="R18" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S18">
+      <c r="S18" s="9">
         <v>2.62</v>
       </c>
-      <c r="T18">
+      <c r="T18" s="9">
         <v>3.91</v>
       </c>
-      <c r="U18">
+      <c r="U18" s="9">
         <v>0.09</v>
       </c>
-      <c r="V18">
+      <c r="V18" s="9">
         <v>99.74</v>
       </c>
-      <c r="W18" t="s">
-        <v>35</v>
-      </c>
-      <c r="X18" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y18" t="s">
+      <c r="W18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y18" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z18" t="s">
+      <c r="Z18" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA18" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB18" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC18" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD18" t="s">
+      <c r="AA18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AD18" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:30">
-      <c r="A19" t="s">
+      <c r="A19" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="2">
         <v>45911</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="8">
         <v>0.45694444444444443</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="9">
         <v>30.553823999999999</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="9">
         <v>-85.935445999999999</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="9">
         <v>30.553823999999999</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="9">
         <v>-85.935445999999999</v>
       </c>
       <c r="I19" t="s">
         <v>39</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="9">
         <v>0.3</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="9">
         <v>21.8</v>
       </c>
-      <c r="L19">
+      <c r="L19" s="9">
         <v>5.38</v>
       </c>
-      <c r="M19">
+      <c r="M19" s="9">
         <v>7.72</v>
       </c>
-      <c r="N19">
+      <c r="N19" s="9">
         <v>88</v>
       </c>
-      <c r="O19">
+      <c r="O19" s="9">
         <v>21.3</v>
       </c>
-      <c r="P19">
+      <c r="P19" s="9">
         <v>0.01</v>
       </c>
-      <c r="Q19">
+      <c r="Q19" s="9">
         <v>3.1</v>
       </c>
-      <c r="R19" t="s">
+      <c r="R19" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S19">
+      <c r="S19" s="9">
         <v>2.62</v>
       </c>
-      <c r="T19">
+      <c r="T19" s="9">
         <v>2.72</v>
       </c>
-      <c r="U19">
+      <c r="U19" s="9">
         <v>0.08</v>
       </c>
-      <c r="V19">
+      <c r="V19" s="9">
         <v>97.4</v>
       </c>
-      <c r="W19" t="s">
-        <v>35</v>
-      </c>
-      <c r="X19" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y19" t="s">
+      <c r="W19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="X19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y19" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="Z19" t="s">
+      <c r="Z19" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AA19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB19" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC19" t="s">
+      <c r="AA19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AC19" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:30">
-      <c r="A20" t="s">
+      <c r="A20" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C20" s="2">
         <v>45911</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="9">
         <v>30.550813999999999</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="9">
         <v>-85.971446999999998</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="9">
         <v>30.550813999999999</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="9">
         <v>-85.971446999999998</v>
       </c>
       <c r="I20" t="s">
         <v>39</v>
       </c>
-      <c r="J20" t="s">
-        <v>42</v>
-      </c>
-      <c r="K20" t="s">
-        <v>42</v>
-      </c>
-      <c r="L20" t="s">
-        <v>42</v>
-      </c>
-      <c r="M20" t="s">
-        <v>42</v>
-      </c>
-      <c r="N20" t="s">
-        <v>42</v>
-      </c>
-      <c r="O20" t="s">
-        <v>42</v>
-      </c>
-      <c r="P20" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>42</v>
-      </c>
-      <c r="R20" t="s">
-        <v>42</v>
-      </c>
-      <c r="S20" t="s">
-        <v>42</v>
-      </c>
-      <c r="T20" t="s">
-        <v>42</v>
-      </c>
-      <c r="U20" t="s">
-        <v>42</v>
-      </c>
-      <c r="V20" t="s">
-        <v>42</v>
-      </c>
-      <c r="W20" t="s">
-        <v>42</v>
-      </c>
-      <c r="X20" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y20" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z20" t="s">
-        <v>42</v>
-      </c>
-      <c r="AA20" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB20" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC20" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD20" t="s">
+      <c r="J20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="L20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="M20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="N20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="O20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="R20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="S20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="T20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="U20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="V20" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="W20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC20" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD20" s="5" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:30">
-      <c r="A21" t="s">
+      <c r="A21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C21" s="2">
         <v>45911</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="9">
         <v>30.543997999999998</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="9">
         <v>-85.958196000000001</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="9">
         <v>30.543997999999998</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="9">
         <v>-85.958196000000001</v>
       </c>
       <c r="I21" t="s">
         <v>39</v>
       </c>
-      <c r="J21" t="s">
-        <v>42</v>
-      </c>
-      <c r="K21" t="s">
-        <v>42</v>
-      </c>
-      <c r="L21" t="s">
-        <v>42</v>
-      </c>
-      <c r="M21" t="s">
-        <v>42</v>
-      </c>
-      <c r="N21" t="s">
-        <v>42</v>
-      </c>
-      <c r="O21" t="s">
-        <v>42</v>
-      </c>
-      <c r="P21" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>42</v>
-      </c>
-      <c r="R21" t="s">
-        <v>42</v>
-      </c>
-      <c r="S21" t="s">
-        <v>42</v>
-      </c>
-      <c r="T21" t="s">
-        <v>42</v>
-      </c>
-      <c r="U21" t="s">
-        <v>42</v>
-      </c>
-      <c r="V21" t="s">
-        <v>42</v>
-      </c>
-      <c r="W21" t="s">
-        <v>42</v>
-      </c>
-      <c r="X21" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y21" t="s">
-        <v>42</v>
-      </c>
-      <c r="Z21" t="s">
-        <v>42</v>
-      </c>
-      <c r="AA21" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB21" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC21" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD21" t="s">
+      <c r="J21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="M21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="O21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="R21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="S21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="T21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="U21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="V21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="W21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="X21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC21" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AD21" s="5" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
edited sites name entries in spreadsheet to match field names in sites_stratv7. no change in standard error estimates when field coordinates used.
</commit_message>
<xml_diff>
--- a/survey_wqdata/SR_Data_editsv2.xlsx
+++ b/survey_wqdata/SR_Data_editsv2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atweg\Documents\Mike\Nokuse\R_sevensrun\nokuse_seven_runs_survey\survey_wqdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADFAE02-DFDF-4877-923B-AC1E4FCADF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF820D8-7BAB-430F-970D-2EB8627836C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
+    <workbookView xWindow="558" yWindow="234" windowWidth="11418" windowHeight="11730" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,36 +33,6 @@
     <t>Site</t>
   </si>
   <si>
-    <t>sr_mst_a</t>
-  </si>
-  <si>
-    <t>sr_mst_b</t>
-  </si>
-  <si>
-    <t>sr_mst_c</t>
-  </si>
-  <si>
-    <t>sr_mst_d</t>
-  </si>
-  <si>
-    <t>sr_mst_e</t>
-  </si>
-  <si>
-    <t>sr_mst_f</t>
-  </si>
-  <si>
-    <t>mck_br_a</t>
-  </si>
-  <si>
-    <t>mck_br_b</t>
-  </si>
-  <si>
-    <t>mck_br_c</t>
-  </si>
-  <si>
-    <t>mck_br_d</t>
-  </si>
-  <si>
     <t>sm_br_a</t>
   </si>
   <si>
@@ -232,6 +202,36 @@
   </si>
   <si>
     <t>Canopy_pct</t>
+  </si>
+  <si>
+    <t>mck_a</t>
+  </si>
+  <si>
+    <t>mck_b</t>
+  </si>
+  <si>
+    <t>mck_c</t>
+  </si>
+  <si>
+    <t>mck_d</t>
+  </si>
+  <si>
+    <t>mst_a</t>
+  </si>
+  <si>
+    <t>mst_b</t>
+  </si>
+  <si>
+    <t>mst_c</t>
+  </si>
+  <si>
+    <t>mst_d</t>
+  </si>
+  <si>
+    <t>mst_e</t>
+  </si>
+  <si>
+    <t>mst_f</t>
   </si>
 </sst>
 </file>
@@ -239,7 +239,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -293,8 +293,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -657,99 +657,99 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="J1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="AA1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="AB1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="AC1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="AD1" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC1" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="AD1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:30">
       <c r="A2" s="5" t="s">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C2" s="2">
         <v>45909</v>
@@ -770,7 +770,7 @@
         <v>-86.038640000000001</v>
       </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J2" s="9">
         <v>0.25</v>
@@ -797,7 +797,7 @@
         <v>1.63</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S2" s="9">
         <v>1.37</v>
@@ -812,42 +812,42 @@
         <v>99.48</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB2" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AD2" s="5" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:30">
       <c r="A3" s="5" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C3" s="2">
         <v>45909</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E3" s="9">
         <v>30.574836999999999</v>
@@ -862,7 +862,7 @@
         <v>-86.028282000000004</v>
       </c>
       <c r="I3" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J3" s="9">
         <v>0.38</v>
@@ -889,7 +889,7 @@
         <v>2.56</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S3" s="9">
         <v>2.69</v>
@@ -904,33 +904,33 @@
         <v>95.84</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA3" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC3" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:30">
       <c r="A4" s="5" t="s">
-        <v>3</v>
+        <v>64</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2">
         <v>45909</v>
@@ -951,7 +951,7 @@
         <v>-86.016197000000005</v>
       </c>
       <c r="I4" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J4" s="9">
         <v>0.4</v>
@@ -978,7 +978,7 @@
         <v>2.14</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S4" s="9">
         <v>4.83</v>
@@ -993,36 +993,36 @@
         <v>99.48</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y4" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z4" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA4" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB4" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC4" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AD4" s="5" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:30">
       <c r="A5" s="5" t="s">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2">
         <v>45912</v>
@@ -1043,7 +1043,7 @@
         <v>-85.978043</v>
       </c>
       <c r="I5" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J5" s="9">
         <v>0.32</v>
@@ -1070,7 +1070,7 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S5" s="9">
         <v>6.45</v>
@@ -1085,39 +1085,39 @@
         <v>84.92</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X5" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y5" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z5" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA5" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC5" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:30">
       <c r="A6" s="5" t="s">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2">
         <v>45911</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E6" s="9">
         <v>30.556989999999999</v>
@@ -1132,7 +1132,7 @@
         <v>-85.963860999999994</v>
       </c>
       <c r="I6" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J6" s="9">
         <v>0.32</v>
@@ -1159,7 +1159,7 @@
         <v>3.71</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S6" s="9">
         <v>5.13</v>
@@ -1174,33 +1174,33 @@
         <v>96.1</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA6" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB6" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC6" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:30">
       <c r="A7" s="5" t="s">
-        <v>6</v>
+        <v>67</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C7" s="2">
         <v>45911</v>
@@ -1221,7 +1221,7 @@
         <v>-85.962569000000002</v>
       </c>
       <c r="I7" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J7" s="9">
         <v>0.43</v>
@@ -1248,7 +1248,7 @@
         <v>2.33</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S7" s="9">
         <v>4.83</v>
@@ -1263,33 +1263,33 @@
         <v>92.72</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X7" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y7" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z7" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA7" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB7" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC7" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:30">
       <c r="A8" s="5" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2">
         <v>45910</v>
@@ -1310,7 +1310,7 @@
         <v>-85.979388999999998</v>
       </c>
       <c r="I8" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J8" s="9">
         <v>0.32</v>
@@ -1337,7 +1337,7 @@
         <v>1.44</v>
       </c>
       <c r="R8" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S8" s="9">
         <v>1.65</v>
@@ -1352,33 +1352,33 @@
         <v>97.92</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X8" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z8" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA8" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB8" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC8" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:30">
       <c r="A9" s="5" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C9" s="2">
         <v>45910</v>
@@ -1399,7 +1399,7 @@
         <v>-85.979889</v>
       </c>
       <c r="I9" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J9" s="9">
         <v>0.25</v>
@@ -1426,7 +1426,7 @@
         <v>1.74</v>
       </c>
       <c r="R9" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S9" s="9">
         <v>1.0900000000000001</v>
@@ -1441,33 +1441,33 @@
         <v>100</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X9" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y9" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z9" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA9" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB9" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC9" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:30">
       <c r="A10" s="5" t="s">
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C10" s="2">
         <v>45910</v>
@@ -1488,7 +1488,7 @@
         <v>-85.979528000000002</v>
       </c>
       <c r="I10" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J10" s="9">
         <v>0.25</v>
@@ -1515,7 +1515,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="R10" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S10" s="9">
         <v>2.82</v>
@@ -1530,42 +1530,42 @@
         <v>98.18</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X10" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y10" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z10" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA10" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB10" s="5" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="AC10" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AD10" s="5" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:30">
       <c r="A11" s="5" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C11" s="2">
         <v>45910</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E11" s="9">
         <v>30.567005999999999</v>
@@ -1581,7 +1581,7 @@
         <v>-85.97851</v>
       </c>
       <c r="I11" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J11" s="9">
         <v>0.34</v>
@@ -1608,7 +1608,7 @@
         <v>3.08</v>
       </c>
       <c r="R11" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S11" s="9">
         <v>2.11</v>
@@ -1623,36 +1623,36 @@
         <v>98.44</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X11" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y11" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z11" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA11" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB11" s="5" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="AC11" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AD11" s="5" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:30">
       <c r="A12" s="5" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C12" s="2">
         <v>45910</v>
@@ -1673,7 +1673,7 @@
         <v>-85.965056000000004</v>
       </c>
       <c r="I12" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J12" s="9">
         <v>0.23</v>
@@ -1700,7 +1700,7 @@
         <v>2</v>
       </c>
       <c r="R12" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S12" s="9">
         <v>1.4</v>
@@ -1715,33 +1715,33 @@
         <v>99.22</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X12" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y12" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z12" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA12" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB12" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC12" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:30">
       <c r="A13" s="5" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C13" s="2">
         <v>45910</v>
@@ -1762,7 +1762,7 @@
         <v>-85.966333000000006</v>
       </c>
       <c r="I13" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J13" s="9">
         <v>0.31</v>
@@ -1789,7 +1789,7 @@
         <v>2.48</v>
       </c>
       <c r="R13" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S13" s="9">
         <v>2.74</v>
@@ -1804,33 +1804,33 @@
         <v>99.48</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X13" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y13" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z13" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA13" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB13" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC13" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:30">
       <c r="A14" s="5" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C14" s="2">
         <v>45911</v>
@@ -1851,7 +1851,7 @@
         <v>-85.966443999999996</v>
       </c>
       <c r="I14" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J14" s="9">
         <v>0.3</v>
@@ -1878,7 +1878,7 @@
         <v>1.85</v>
       </c>
       <c r="R14" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S14" s="9">
         <v>2.62</v>
@@ -1893,33 +1893,33 @@
         <v>97.66</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X14" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y14" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z14" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA14" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB14" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC14" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:30">
       <c r="A15" s="5" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C15" s="2">
         <v>45912</v>
@@ -1937,78 +1937,78 @@
         <v>-85.984607999999994</v>
       </c>
       <c r="I15" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="O15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Q15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="R15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="T15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="U15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="V15" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="X15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Y15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Z15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AA15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AB15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AC15" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AD15" s="5" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:30">
       <c r="A16" s="5" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C16" s="2">
         <v>45912</v>
@@ -2029,7 +2029,7 @@
         <v>-85.981594000000001</v>
       </c>
       <c r="I16" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J16" s="9">
         <v>0.22</v>
@@ -2056,7 +2056,7 @@
         <v>3.51</v>
       </c>
       <c r="R16" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S16" s="9">
         <v>2.72</v>
@@ -2071,33 +2071,33 @@
         <v>98.18</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X16" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y16" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z16" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA16" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB16" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC16" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:30">
       <c r="A17" s="5" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C17" s="2">
         <v>45911</v>
@@ -2118,78 +2118,78 @@
         <v>-85.919370000000001</v>
       </c>
       <c r="I17" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="R17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="S17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="T17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="U17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="V17" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="X17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Y17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Z17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AA17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AB17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AC17" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AD17" s="5" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:30">
       <c r="A18" s="5" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C18" s="2">
         <v>45909</v>
@@ -2210,7 +2210,7 @@
         <v>-85.999088</v>
       </c>
       <c r="I18" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J18" s="9">
         <v>0.36</v>
@@ -2237,7 +2237,7 @@
         <v>2.82</v>
       </c>
       <c r="R18" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S18" s="9">
         <v>2.62</v>
@@ -2252,36 +2252,36 @@
         <v>99.74</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X18" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y18" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z18" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA18" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB18" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC18" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AD18" s="5" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:30">
       <c r="A19" s="5" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C19" s="2">
         <v>45911</v>
@@ -2302,7 +2302,7 @@
         <v>-85.935445999999999</v>
       </c>
       <c r="I19" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J19" s="9">
         <v>0.3</v>
@@ -2329,7 +2329,7 @@
         <v>3.1</v>
       </c>
       <c r="R19" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="S19" s="9">
         <v>2.62</v>
@@ -2344,33 +2344,33 @@
         <v>97.4</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="X19" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Y19" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="Z19" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA19" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AB19" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AC19" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:30">
       <c r="A20" s="5" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C20" s="2">
         <v>45911</v>
@@ -2388,78 +2388,78 @@
         <v>-85.971446999999998</v>
       </c>
       <c r="I20" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="M20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="N20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="O20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="P20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Q20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="R20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="S20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="T20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="U20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="V20" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="X20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Y20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Z20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AA20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AB20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AC20" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AD20" s="5" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:30">
       <c r="A21" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C21" s="2">
         <v>45911</v>
@@ -2477,70 +2477,70 @@
         <v>-85.958196000000001</v>
       </c>
       <c r="I21" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Q21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="R21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="S21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="T21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="U21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="V21" s="9" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="X21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Y21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="Z21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AA21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AB21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AC21" s="5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="AD21" s="5" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>